<commit_message>
Updated Weekly Daily Activity Log
</commit_message>
<xml_diff>
--- a/12609520_CAP776.xlsx
+++ b/12609520_CAP776.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/EE903CDAF4BD63AF/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="363" documentId="8_{E56A0022-F18E-4A5A-8A01-B56BFC90E4AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0878FA74-7E22-4DE9-8ADF-A4A2806032C1}"/>
+  <xr:revisionPtr revIDLastSave="466" documentId="8_{E56A0022-F18E-4A5A-8A01-B56BFC90E4AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9562D0F3-ABDA-4A86-8AB7-CCEACA2042C6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="74">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -223,16 +223,10 @@
     <t xml:space="preserve"> Felt a bit tired after evening class.</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
     <t>High</t>
   </si>
   <si>
     <t>Weekwnd/holiday; sef-study and coding.</t>
-  </si>
-  <si>
-    <t>yes</t>
   </si>
   <si>
     <t>University day; Attended all classes.</t>
@@ -245,6 +239,24 @@
   </si>
   <si>
     <t>Univesity Day; Atteneded all Classes</t>
+  </si>
+  <si>
+    <t>Attended Tuesday classes; revised practical work and completed codding practice.</t>
+  </si>
+  <si>
+    <t>Heavy University Day; Attended all Classes and  practiced coding afterward.</t>
+  </si>
+  <si>
+    <t>Attended Thursday classes; revised practical work and completed codding practice.</t>
+  </si>
+  <si>
+    <t>statisfied</t>
+  </si>
+  <si>
+    <t>Sunday holiday; revised coursework and practiced python independently.</t>
+  </si>
+  <si>
+    <t>Saturday holiday; spent extra time studying and working on coding exercieses.</t>
   </si>
 </sst>
 </file>
@@ -1252,8 +1264,8 @@
       <c r="F10" s="14">
         <v>0</v>
       </c>
-      <c r="G10" s="14" t="s">
-        <v>62</v>
+      <c r="G10" s="14">
+        <v>0</v>
       </c>
       <c r="H10" s="14">
         <v>250</v>
@@ -1272,10 +1284,10 @@
         <v>50</v>
       </c>
       <c r="M10" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N10" s="17" t="s">
         <v>63</v>
-      </c>
-      <c r="N10" s="17" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
@@ -1297,8 +1309,8 @@
       <c r="F11" s="14">
         <v>0</v>
       </c>
-      <c r="G11" s="14" t="s">
-        <v>62</v>
+      <c r="G11" s="14">
+        <v>0</v>
       </c>
       <c r="H11" s="14">
         <v>250</v>
@@ -1317,10 +1329,10 @@
         <v>50</v>
       </c>
       <c r="M11" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N11" s="17" t="s">
         <v>63</v>
-      </c>
-      <c r="N11" s="17" t="s">
-        <v>64</v>
       </c>
       <c r="O11" t="s">
         <v>57</v>
@@ -1345,8 +1357,8 @@
       <c r="F12" s="14">
         <v>300</v>
       </c>
-      <c r="G12" s="14" t="s">
-        <v>65</v>
+      <c r="G12" s="14">
+        <v>6</v>
       </c>
       <c r="H12" s="14">
         <v>250</v>
@@ -1368,7 +1380,7 @@
         <v>51</v>
       </c>
       <c r="N12" s="17" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
@@ -1390,8 +1402,8 @@
       <c r="F13" s="14">
         <v>200</v>
       </c>
-      <c r="G13" s="14" t="s">
-        <v>65</v>
+      <c r="G13" s="14">
+        <v>4</v>
       </c>
       <c r="H13" s="14">
         <v>250</v>
@@ -1413,7 +1425,7 @@
         <v>51</v>
       </c>
       <c r="N13" s="17" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
@@ -1435,8 +1447,8 @@
       <c r="F14" s="14">
         <v>400</v>
       </c>
-      <c r="G14" s="14" t="s">
-        <v>65</v>
+      <c r="G14" s="14">
+        <v>8</v>
       </c>
       <c r="H14" s="14">
         <v>250</v>
@@ -1449,7 +1461,7 @@
         <v>305</v>
       </c>
       <c r="K14" s="16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L14" s="16" t="s">
         <v>50</v>
@@ -1458,7 +1470,7 @@
         <v>59</v>
       </c>
       <c r="N14" s="17" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
@@ -1480,8 +1492,8 @@
       <c r="F15" s="14">
         <v>200</v>
       </c>
-      <c r="G15" s="14" t="s">
-        <v>65</v>
+      <c r="G15" s="14">
+        <v>4</v>
       </c>
       <c r="H15" s="14">
         <v>250</v>
@@ -1503,7 +1515,7 @@
         <v>51</v>
       </c>
       <c r="N15" s="17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
@@ -1525,8 +1537,8 @@
       <c r="F16" s="14">
         <v>250</v>
       </c>
-      <c r="G16" s="14" t="s">
-        <v>65</v>
+      <c r="G16" s="14">
+        <v>5</v>
       </c>
       <c r="H16" s="14">
         <v>250</v>
@@ -1548,7 +1560,7 @@
         <v>51</v>
       </c>
       <c r="N16" s="17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1570,8 +1582,8 @@
       <c r="F17" s="14">
         <v>0</v>
       </c>
-      <c r="G17" s="14" t="s">
-        <v>62</v>
+      <c r="G17" s="14">
+        <v>0</v>
       </c>
       <c r="H17" s="14">
         <v>250</v>
@@ -1590,10 +1602,10 @@
         <v>50</v>
       </c>
       <c r="M17" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N17" s="17" t="s">
         <v>63</v>
-      </c>
-      <c r="N17" s="17" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1615,8 +1627,8 @@
       <c r="F18" s="14">
         <v>0</v>
       </c>
-      <c r="G18" s="14" t="s">
-        <v>62</v>
+      <c r="G18" s="14">
+        <v>0</v>
       </c>
       <c r="H18" s="14">
         <v>250</v>
@@ -1635,10 +1647,10 @@
         <v>50</v>
       </c>
       <c r="M18" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N18" s="17" t="s">
         <v>63</v>
-      </c>
-      <c r="N18" s="17" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1660,8 +1672,8 @@
       <c r="F19" s="14">
         <v>300</v>
       </c>
-      <c r="G19" s="14" t="s">
-        <v>65</v>
+      <c r="G19" s="14">
+        <v>6</v>
       </c>
       <c r="H19" s="14">
         <v>250</v>
@@ -1683,7 +1695,7 @@
         <v>51</v>
       </c>
       <c r="N19" s="17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1705,8 +1717,8 @@
       <c r="F20" s="14">
         <v>200</v>
       </c>
-      <c r="G20" s="14" t="s">
-        <v>65</v>
+      <c r="G20" s="14">
+        <v>4</v>
       </c>
       <c r="H20" s="14">
         <v>250</v>
@@ -1728,7 +1740,7 @@
         <v>51</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1750,8 +1762,8 @@
       <c r="F21" s="14">
         <v>400</v>
       </c>
-      <c r="G21" s="14" t="s">
-        <v>65</v>
+      <c r="G21" s="14">
+        <v>8</v>
       </c>
       <c r="H21" s="14">
         <v>250</v>
@@ -1764,7 +1776,7 @@
         <v>245</v>
       </c>
       <c r="K21" s="16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L21" s="16" t="s">
         <v>50</v>
@@ -1773,7 +1785,7 @@
         <v>59</v>
       </c>
       <c r="N21" s="17" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1795,8 +1807,8 @@
       <c r="F22" s="14">
         <v>200</v>
       </c>
-      <c r="G22" s="14" t="s">
-        <v>65</v>
+      <c r="G22" s="14">
+        <v>4</v>
       </c>
       <c r="H22" s="14">
         <v>250</v>
@@ -1818,7 +1830,7 @@
         <v>51</v>
       </c>
       <c r="N22" s="17" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1840,8 +1852,8 @@
       <c r="F23" s="14">
         <v>250</v>
       </c>
-      <c r="G23" s="14" t="s">
-        <v>65</v>
+      <c r="G23" s="14">
+        <v>5</v>
       </c>
       <c r="H23" s="14">
         <v>250</v>
@@ -1863,7 +1875,7 @@
         <v>51</v>
       </c>
       <c r="N23" s="17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1885,8 +1897,8 @@
       <c r="F24" s="14">
         <v>0</v>
       </c>
-      <c r="G24" s="14" t="s">
-        <v>62</v>
+      <c r="G24" s="14">
+        <v>0</v>
       </c>
       <c r="H24" s="14">
         <v>250</v>
@@ -1905,10 +1917,10 @@
         <v>50</v>
       </c>
       <c r="M24" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N24" s="17" t="s">
         <v>63</v>
-      </c>
-      <c r="N24" s="17" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1930,8 +1942,8 @@
       <c r="F25" s="14">
         <v>0</v>
       </c>
-      <c r="G25" s="14" t="s">
-        <v>62</v>
+      <c r="G25" s="14">
+        <v>0</v>
       </c>
       <c r="H25" s="14">
         <v>250</v>
@@ -1950,10 +1962,10 @@
         <v>50</v>
       </c>
       <c r="M25" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N25" s="17" t="s">
         <v>63</v>
-      </c>
-      <c r="N25" s="17" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1975,8 +1987,8 @@
       <c r="F26" s="14">
         <v>300</v>
       </c>
-      <c r="G26" s="14" t="s">
-        <v>65</v>
+      <c r="G26" s="14">
+        <v>6</v>
       </c>
       <c r="H26" s="14">
         <v>250</v>
@@ -1998,143 +2010,288 @@
         <v>51</v>
       </c>
       <c r="N26" s="17" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="13">
+        <v>46273</v>
+      </c>
+      <c r="B27" s="14">
+        <v>420</v>
+      </c>
+      <c r="C27" s="14">
+        <v>30</v>
+      </c>
+      <c r="D27" s="14">
+        <v>20</v>
+      </c>
+      <c r="E27" s="14">
+        <v>75</v>
+      </c>
+      <c r="F27" s="14">
+        <v>200</v>
+      </c>
+      <c r="G27" s="14">
+        <v>4</v>
+      </c>
+      <c r="H27" s="14">
+        <v>250</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>995</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="17"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+        <v>445</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="13">
+        <v>46274</v>
+      </c>
+      <c r="B28" s="14">
+        <v>390</v>
+      </c>
+      <c r="C28" s="14">
+        <v>30</v>
+      </c>
+      <c r="D28" s="14">
+        <v>20</v>
+      </c>
+      <c r="E28" s="14">
+        <v>75</v>
+      </c>
+      <c r="F28" s="14">
+        <v>400</v>
+      </c>
+      <c r="G28" s="14">
+        <v>8</v>
+      </c>
+      <c r="H28" s="14">
+        <v>250</v>
+      </c>
+      <c r="I28" s="15">
+        <v>1135</v>
+      </c>
+      <c r="J28" s="15">
+        <f t="shared" si="0"/>
+        <v>305</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B29" s="14">
+        <v>390</v>
+      </c>
+      <c r="C29" s="14">
+        <v>30</v>
+      </c>
+      <c r="D29" s="14">
+        <v>20</v>
+      </c>
+      <c r="E29" s="14">
+        <v>75</v>
+      </c>
+      <c r="F29" s="14">
+        <v>200</v>
+      </c>
+      <c r="G29" s="14">
+        <v>4</v>
+      </c>
+      <c r="H29" s="14">
+        <v>250</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>965</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+        <v>475</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A30" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B30" s="14">
+        <v>420</v>
+      </c>
+      <c r="C30" s="14">
+        <v>30</v>
+      </c>
+      <c r="D30" s="14">
+        <v>20</v>
+      </c>
+      <c r="E30" s="14">
+        <v>75</v>
+      </c>
+      <c r="F30" s="14">
+        <v>250</v>
+      </c>
+      <c r="G30" s="14">
+        <v>5</v>
+      </c>
+      <c r="H30" s="14">
+        <v>250</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>1045</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="17"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+        <v>395</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="13">
+        <v>46277</v>
+      </c>
+      <c r="B31" s="14">
+        <v>390</v>
+      </c>
+      <c r="C31" s="14">
+        <v>30</v>
+      </c>
+      <c r="D31" s="14">
+        <v>120</v>
+      </c>
+      <c r="E31" s="14">
+        <v>120</v>
+      </c>
+      <c r="F31" s="14">
+        <v>0</v>
+      </c>
+      <c r="G31" s="14">
+        <v>0</v>
+      </c>
+      <c r="H31" s="14">
+        <v>250</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>910</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="17"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+        <v>530</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N31" s="17" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="13">
+        <v>46278</v>
+      </c>
+      <c r="B32" s="14">
+        <v>390</v>
+      </c>
+      <c r="C32" s="14">
+        <v>30</v>
+      </c>
+      <c r="D32" s="14">
+        <v>120</v>
+      </c>
+      <c r="E32" s="14">
+        <v>120</v>
+      </c>
+      <c r="F32" s="14">
+        <v>0</v>
+      </c>
+      <c r="G32" s="14">
+        <v>0</v>
+      </c>
+      <c r="H32" s="14">
+        <v>250</v>
+      </c>
+      <c r="I32" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>910</v>
+      </c>
+      <c r="J32" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="17"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="13"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J32" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="17"/>
+        <v>530</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L32" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M32" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N32" s="17" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="13"/>
+      <c r="A33" s="13">
+        <v>46279</v>
+      </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
       <c r="D33" s="14"/>

</xml_diff>